<commit_message>
KPI actualizado 2026-08-10 20:56 UTC
</commit_message>
<xml_diff>
--- a/data/50001504 - ZITRON PERU CODESTABLE A.xlsx
+++ b/data/50001504 - ZITRON PERU CODESTABLE A.xlsx
@@ -1431,13 +1431,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46077.51147570602</v>
+        <v>46077.34480903935</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.72374829861</v>
+        <v>46092.557081631945</v>
       </c>
       <c r="D4" s="5">
-        <v>46118.784329155096</v>
+        <v>46118.617662488425</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1482,13 +1482,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46077.51154885416</v>
+        <v>46077.3448821875</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.723712962965</v>
+        <v>46092.55704629629</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.901517754624</v>
+        <v>46133.73485108797</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1547,13 +1547,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46077.511553495366</v>
+        <v>46077.34488682871</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.723713495376</v>
+        <v>46092.557046828704</v>
       </c>
       <c r="D6" s="5">
-        <v>46100.64636372685</v>
+        <v>46100.47969706019</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1612,13 +1612,13 @@
         <v>39</v>
       </c>
       <c r="B7" s="8">
-        <v>46077.511557418984</v>
+        <v>46077.34489075231</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.723713935186</v>
+        <v>46092.55704726852</v>
       </c>
       <c r="D7" s="8">
-        <v>46226.564140381946</v>
+        <v>46226.397473715275</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>40</v>
@@ -1677,13 +1677,13 @@
         <v>42</v>
       </c>
       <c r="B8" s="5">
-        <v>46077.51156111111</v>
+        <v>46077.344894444446</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.7237144213</v>
+        <v>46092.55704775463</v>
       </c>
       <c r="D8" s="5">
-        <v>46100.69251282407</v>
+        <v>46100.52584615741</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>43</v>
@@ -1742,13 +1742,13 @@
         <v>46</v>
       </c>
       <c r="B9" s="8">
-        <v>46077.51156568287</v>
+        <v>46077.3448990162</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.723715127315</v>
+        <v>46092.55704846064</v>
       </c>
       <c r="D9" s="8">
-        <v>46100.67660435185</v>
+        <v>46100.50993768519</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>47</v>
@@ -1807,13 +1807,13 @@
         <v>49</v>
       </c>
       <c r="B10" s="5">
-        <v>46077.511480243054</v>
+        <v>46077.34481357639</v>
       </c>
       <c r="C10" s="5">
-        <v>46114.52695974537</v>
+        <v>46114.3602930787</v>
       </c>
       <c r="D10" s="5">
-        <v>46114.52697136574</v>
+        <v>46114.360304699076</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>50</v>
@@ -1860,13 +1860,13 @@
         <v>52</v>
       </c>
       <c r="B11" s="8">
-        <v>46077.51157018519</v>
+        <v>46077.34490351852</v>
       </c>
       <c r="C11" s="8">
-        <v>46100.64395409722</v>
+        <v>46100.477287430556</v>
       </c>
       <c r="D11" s="8">
-        <v>46100.643973819446</v>
+        <v>46100.477307152774</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>53</v>
@@ -1925,13 +1925,13 @@
         <v>56</v>
       </c>
       <c r="B12" s="5">
-        <v>46077.5115900463</v>
+        <v>46077.34492337963</v>
       </c>
       <c r="C12" s="5">
-        <v>46100.644285208335</v>
+        <v>46100.47761854167</v>
       </c>
       <c r="D12" s="5">
-        <v>46100.690858877315</v>
+        <v>46100.52419221065</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -1990,13 +1990,13 @@
         <v>60</v>
       </c>
       <c r="B13" s="8">
-        <v>46077.511595937496</v>
+        <v>46077.34492927083</v>
       </c>
       <c r="C13" s="8">
-        <v>46097.53360980324</v>
+        <v>46097.36694313657</v>
       </c>
       <c r="D13" s="8">
-        <v>46101.819566875</v>
+        <v>46101.65290020833</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>61</v>
@@ -2055,13 +2055,13 @@
         <v>64</v>
       </c>
       <c r="B14" s="5">
-        <v>46077.51160226852</v>
+        <v>46077.344935601854</v>
       </c>
       <c r="C14" s="5">
-        <v>46114.5269425</v>
+        <v>46114.36027583333</v>
       </c>
       <c r="D14" s="5">
-        <v>46114.526961006944</v>
+        <v>46114.36029434028</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>65</v>
@@ -2120,13 +2120,13 @@
         <v>68</v>
       </c>
       <c r="B15" s="8">
-        <v>46077.51148475695</v>
+        <v>46077.34481809028</v>
       </c>
       <c r="C15" s="8">
-        <v>46100.65183821759</v>
+        <v>46100.48517155093</v>
       </c>
       <c r="D15" s="8">
-        <v>46100.6518556713</v>
+        <v>46100.48518900463</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>69</v>
@@ -2173,13 +2173,13 @@
         <v>71</v>
       </c>
       <c r="B16" s="5">
-        <v>46077.51161194444</v>
+        <v>46077.34494527778</v>
       </c>
       <c r="C16" s="5">
-        <v>46100.6514</v>
+        <v>46100.48473333333</v>
       </c>
       <c r="D16" s="5">
-        <v>46181.66261890046</v>
+        <v>46181.495952233796</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>72</v>
@@ -2238,13 +2238,13 @@
         <v>75</v>
       </c>
       <c r="B17" s="8">
-        <v>46077.511618379634</v>
+        <v>46077.34495171296</v>
       </c>
       <c r="C17" s="8">
-        <v>46100.65097256945</v>
+        <v>46100.48430590278</v>
       </c>
       <c r="D17" s="8">
-        <v>46100.65176030093</v>
+        <v>46100.485093634255</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>76</v>
@@ -2303,13 +2303,13 @@
         <v>78</v>
       </c>
       <c r="B18" s="5">
-        <v>46077.511624872684</v>
+        <v>46077.34495820602</v>
       </c>
       <c r="C18" s="5">
-        <v>46100.651822280095</v>
+        <v>46100.48515561342</v>
       </c>
       <c r="D18" s="5">
-        <v>46223.81906920139</v>
+        <v>46223.65240253472</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>79</v>
@@ -2368,13 +2368,13 @@
         <v>84</v>
       </c>
       <c r="B19" s="8">
-        <v>46077.511631180554</v>
+        <v>46077.34496451389</v>
       </c>
       <c r="C19" s="8">
-        <v>46097.53366215278</v>
+        <v>46097.36699548611</v>
       </c>
       <c r="D19" s="8">
-        <v>46223.81906576389</v>
+        <v>46223.65239909722</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>85</v>
@@ -2433,13 +2433,13 @@
         <v>88</v>
       </c>
       <c r="B20" s="5">
-        <v>46077.511489247685</v>
+        <v>46077.34482258101</v>
       </c>
       <c r="C20" s="5">
-        <v>46181.58434533565</v>
+        <v>46181.41767866898</v>
       </c>
       <c r="D20" s="5">
-        <v>46228.464923321764</v>
+        <v>46228.29825665509</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>89</v>
@@ -2482,13 +2482,13 @@
         <v>91</v>
       </c>
       <c r="B21" s="8">
-        <v>46077.511642847225</v>
+        <v>46077.34497618055</v>
       </c>
       <c r="C21" s="8">
-        <v>46104.59183936343</v>
+        <v>46104.42517269676</v>
       </c>
       <c r="D21" s="8">
-        <v>46104.59185236111</v>
+        <v>46104.42518569445</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>92</v>
@@ -2547,13 +2547,13 @@
         <v>97</v>
       </c>
       <c r="B22" s="5">
-        <v>46077.51164822916</v>
+        <v>46077.3449815625</v>
       </c>
       <c r="C22" s="5">
-        <v>46104.59146888889</v>
+        <v>46104.424802222224</v>
       </c>
       <c r="D22" s="5">
-        <v>46104.59147082176</v>
+        <v>46104.42480415509</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>98</v>
@@ -2608,13 +2608,13 @@
         <v>102</v>
       </c>
       <c r="B23" s="8">
-        <v>46077.51165403935</v>
+        <v>46077.344987372686</v>
       </c>
       <c r="C23" s="8">
-        <v>46104.59182263889</v>
+        <v>46104.42515597222</v>
       </c>
       <c r="D23" s="8">
-        <v>46104.59182434028</v>
+        <v>46104.42515767361</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>103</v>
@@ -2669,13 +2669,13 @@
         <v>105</v>
       </c>
       <c r="B24" s="5">
-        <v>46077.51165996528</v>
+        <v>46077.34499329861</v>
       </c>
       <c r="C24" s="5">
-        <v>46104.59360127315</v>
+        <v>46104.42693460648</v>
       </c>
       <c r="D24" s="5">
-        <v>46104.593614618054</v>
+        <v>46104.42694795139</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>106</v>
@@ -2734,13 +2734,13 @@
         <v>108</v>
       </c>
       <c r="B25" s="8">
-        <v>46077.51166581019</v>
+        <v>46077.34499914352</v>
       </c>
       <c r="C25" s="8">
-        <v>46104.59354353009</v>
+        <v>46104.42687686342</v>
       </c>
       <c r="D25" s="8">
-        <v>46104.59354552084</v>
+        <v>46104.42687885417</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>109</v>
@@ -2795,13 +2795,13 @@
         <v>111</v>
       </c>
       <c r="B26" s="5">
-        <v>46077.51167158565</v>
+        <v>46077.345004918985</v>
       </c>
       <c r="C26" s="5">
-        <v>46104.59358512731</v>
+        <v>46104.42691846065</v>
       </c>
       <c r="D26" s="5">
-        <v>46104.59358693287</v>
+        <v>46104.4269202662</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>112</v>
@@ -2856,13 +2856,13 @@
         <v>114</v>
       </c>
       <c r="B27" s="8">
-        <v>46077.5116772801</v>
+        <v>46077.345010613426</v>
       </c>
       <c r="C27" s="8">
-        <v>46174.61983740741</v>
+        <v>46174.453170740744</v>
       </c>
       <c r="D27" s="8">
-        <v>46181.6626696875</v>
+        <v>46181.49600302083</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>115</v>
@@ -2921,13 +2921,13 @@
         <v>118</v>
       </c>
       <c r="B28" s="5">
-        <v>46077.51173550926</v>
+        <v>46077.345068842595</v>
       </c>
       <c r="C28" s="5">
-        <v>46104.5946865625</v>
+        <v>46104.42801989583</v>
       </c>
       <c r="D28" s="5">
-        <v>46104.59468819444</v>
+        <v>46104.42802152778</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>119</v>
@@ -2982,13 +2982,13 @@
         <v>121</v>
       </c>
       <c r="B29" s="8">
-        <v>46077.51174407407</v>
+        <v>46077.34507740741</v>
       </c>
       <c r="C29" s="8">
-        <v>46174.61930413195</v>
+        <v>46174.45263746528</v>
       </c>
       <c r="D29" s="8">
-        <v>46174.619306099536</v>
+        <v>46174.45263943287</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>122</v>
@@ -3043,13 +3043,13 @@
         <v>124</v>
       </c>
       <c r="B30" s="5">
-        <v>46077.511750624995</v>
+        <v>46077.34508395834</v>
       </c>
       <c r="C30" s="5">
-        <v>46127.78436329861</v>
+        <v>46127.61769663195</v>
       </c>
       <c r="D30" s="5">
-        <v>46127.7843647338</v>
+        <v>46127.61769806713</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>125</v>
@@ -3104,13 +3104,13 @@
         <v>127</v>
       </c>
       <c r="B31" s="8">
-        <v>46077.511757326385</v>
+        <v>46077.34509065972</v>
       </c>
       <c r="C31" s="8">
-        <v>46104.59300746528</v>
+        <v>46104.426340798615</v>
       </c>
       <c r="D31" s="8">
-        <v>46104.593021875</v>
+        <v>46104.42635520833</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>128</v>
@@ -3169,13 +3169,13 @@
         <v>132</v>
       </c>
       <c r="B32" s="5">
-        <v>46077.51176472222</v>
+        <v>46077.34509805556</v>
       </c>
       <c r="C32" s="5">
-        <v>46097.53370762731</v>
+        <v>46097.36704096065</v>
       </c>
       <c r="D32" s="5">
-        <v>46097.53370961806</v>
+        <v>46097.36704295139</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>133</v>
@@ -3230,13 +3230,13 @@
         <v>135</v>
       </c>
       <c r="B33" s="8">
-        <v>46077.511778726854</v>
+        <v>46077.34511206018</v>
       </c>
       <c r="C33" s="8">
-        <v>46104.59299090278</v>
+        <v>46104.42632423611</v>
       </c>
       <c r="D33" s="8">
-        <v>46104.59299259259</v>
+        <v>46104.426325925924</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>136</v>
@@ -3291,13 +3291,13 @@
         <v>138</v>
       </c>
       <c r="B34" s="5">
-        <v>46077.511493680555</v>
+        <v>46077.34482701389</v>
       </c>
       <c r="C34" s="5">
-        <v>46181.58435664352</v>
+        <v>46181.41768997685</v>
       </c>
       <c r="D34" s="5">
-        <v>46181.66279681713</v>
+        <v>46181.496130150466</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>139</v>
@@ -3340,13 +3340,13 @@
         <v>141</v>
       </c>
       <c r="B35" s="8">
-        <v>46077.511804884256</v>
+        <v>46077.34513821759</v>
       </c>
       <c r="C35" s="8">
-        <v>46098.5182991551</v>
+        <v>46098.351632488426</v>
       </c>
       <c r="D35" s="8">
-        <v>46098.51831884259</v>
+        <v>46098.35165217593</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>142</v>
@@ -3405,13 +3405,13 @@
         <v>146</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.511813819445</v>
+        <v>46077.34514715278</v>
       </c>
       <c r="C36" s="5">
-        <v>46132.59997896991</v>
+        <v>46132.43331230324</v>
       </c>
       <c r="D36" s="5">
-        <v>46132.59999503472</v>
+        <v>46132.43332836806</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>147</v>
@@ -3470,13 +3470,13 @@
         <v>150</v>
       </c>
       <c r="B37" s="8">
-        <v>46092.51508778935</v>
+        <v>46092.34842112269</v>
       </c>
       <c r="C37" s="8">
-        <v>46132.600021226855</v>
+        <v>46132.433354560184</v>
       </c>
       <c r="D37" s="8">
-        <v>46132.60003634259</v>
+        <v>46132.43336967593</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>151</v>
@@ -3535,13 +3535,13 @@
         <v>153</v>
       </c>
       <c r="B38" s="5">
-        <v>46092.51515344907</v>
+        <v>46092.34848678241</v>
       </c>
       <c r="C38" s="5">
-        <v>46181.584749965274</v>
+        <v>46181.41808329861</v>
       </c>
       <c r="D38" s="5">
-        <v>46181.66283061342</v>
+        <v>46181.49616394676</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>154</v>
@@ -3600,13 +3600,13 @@
         <v>159</v>
       </c>
       <c r="B39" s="8">
-        <v>46077.511823125</v>
+        <v>46077.34515645834</v>
       </c>
       <c r="C39" s="8">
-        <v>46181.584367777774</v>
+        <v>46181.41770111111</v>
       </c>
       <c r="D39" s="8">
-        <v>46181.58436929398</v>
+        <v>46181.41770262731</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>160</v>
@@ -3649,13 +3649,13 @@
         <v>162</v>
       </c>
       <c r="B40" s="5">
-        <v>46077.51182792824</v>
+        <v>46077.345161261575</v>
       </c>
       <c r="C40" s="5">
-        <v>46181.58420413194</v>
+        <v>46181.41753746528</v>
       </c>
       <c r="D40" s="5">
-        <v>46181.66295334491</v>
+        <v>46181.496286678244</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>163</v>
@@ -3714,13 +3714,13 @@
         <v>167</v>
       </c>
       <c r="B41" s="8">
-        <v>46077.511842673615</v>
+        <v>46077.345176006944</v>
       </c>
       <c r="C41" s="8">
-        <v>46147.535636643515</v>
+        <v>46147.36896997685</v>
       </c>
       <c r="D41" s="8">
-        <v>46181.66295386574</v>
+        <v>46181.49628719907</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>168</v>
@@ -3779,13 +3779,13 @@
         <v>172</v>
       </c>
       <c r="B42" s="5">
-        <v>46077.51184961805</v>
+        <v>46077.345182951394</v>
       </c>
       <c r="C42" s="5">
-        <v>46181.5844128125</v>
+        <v>46181.41774614583</v>
       </c>
       <c r="D42" s="5">
-        <v>46228.228668194446</v>
+        <v>46228.06200152778</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>173</v>
@@ -3828,13 +3828,13 @@
         <v>175</v>
       </c>
       <c r="B43" s="8">
-        <v>46077.511853495365</v>
+        <v>46077.34518682871</v>
       </c>
       <c r="C43" s="8">
-        <v>46128.502038506944</v>
+        <v>46128.33537184028</v>
       </c>
       <c r="D43" s="8">
-        <v>46147.53564614583</v>
+        <v>46147.36897947917</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>176</v>
@@ -3893,13 +3893,13 @@
         <v>180</v>
       </c>
       <c r="B44" s="5">
-        <v>46077.51185981481</v>
+        <v>46077.34519314815</v>
       </c>
       <c r="C44" s="5">
-        <v>46146.591328703704</v>
+        <v>46146.42466203704</v>
       </c>
       <c r="D44" s="5">
-        <v>46181.66309797454</v>
+        <v>46181.49643130787</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>181</v>
@@ -3958,13 +3958,13 @@
         <v>184</v>
       </c>
       <c r="B45" s="8">
-        <v>46077.51186719908</v>
+        <v>46077.34520053241</v>
       </c>
       <c r="C45" s="8">
-        <v>46147.535923564814</v>
+        <v>46147.36925689815</v>
       </c>
       <c r="D45" s="8">
-        <v>46181.663148680556</v>
+        <v>46181.496482013885</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>185</v>
@@ -4023,13 +4023,13 @@
         <v>188</v>
       </c>
       <c r="B46" s="5">
-        <v>46077.51192424769</v>
+        <v>46077.34525758102</v>
       </c>
       <c r="C46" s="5">
-        <v>46181.58443833333</v>
+        <v>46181.41777166667</v>
       </c>
       <c r="D46" s="5">
-        <v>46181.58443959491</v>
+        <v>46181.41777292824</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>160</v>
@@ -4072,13 +4072,13 @@
         <v>190</v>
       </c>
       <c r="B47" s="8">
-        <v>46077.511929189815</v>
+        <v>46077.345262523144</v>
       </c>
       <c r="C47" s="8">
-        <v>46181.58425488426</v>
+        <v>46181.41758821759</v>
       </c>
       <c r="D47" s="8">
-        <v>46181.66326342593</v>
+        <v>46181.49659675926</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>191</v>
@@ -4137,13 +4137,13 @@
         <v>193</v>
       </c>
       <c r="B48" s="5">
-        <v>46077.51193605324</v>
+        <v>46077.34526938657</v>
       </c>
       <c r="C48" s="5">
-        <v>46181.58426366898</v>
+        <v>46181.41759700231</v>
       </c>
       <c r="D48" s="5">
-        <v>46181.663263993054</v>
+        <v>46181.49659732639</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>194</v>
@@ -4202,13 +4202,13 @@
         <v>196</v>
       </c>
       <c r="B49" s="8">
-        <v>46077.51194265047</v>
+        <v>46077.3452759838</v>
       </c>
       <c r="C49" s="8">
-        <v>46181.58426854167</v>
+        <v>46181.417601875</v>
       </c>
       <c r="D49" s="8">
-        <v>46181.66326457176</v>
+        <v>46181.49659790509</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>197</v>
@@ -4267,13 +4267,13 @@
         <v>199</v>
       </c>
       <c r="B50" s="5">
-        <v>46077.511954409725</v>
+        <v>46077.34528774305</v>
       </c>
       <c r="C50" s="5">
-        <v>46181.5858024537</v>
+        <v>46181.41913578704</v>
       </c>
       <c r="D50" s="5">
-        <v>46181.58580350694</v>
+        <v>46181.41913684028</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>200</v>
@@ -4316,13 +4316,13 @@
         <v>202</v>
       </c>
       <c r="B51" s="8">
-        <v>46077.51195832176</v>
+        <v>46077.34529165509</v>
       </c>
       <c r="C51" s="8">
-        <v>46181.58428013889</v>
+        <v>46181.41761347222</v>
       </c>
       <c r="D51" s="8">
-        <v>46223.8191834375</v>
+        <v>46223.65251677083</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>203</v>
@@ -4381,13 +4381,13 @@
         <v>205</v>
       </c>
       <c r="B52" s="5">
-        <v>46077.511964687495</v>
+        <v>46077.34529802084</v>
       </c>
       <c r="C52" s="5">
-        <v>46181.584470057875</v>
+        <v>46181.4178033912</v>
       </c>
       <c r="D52" s="5">
-        <v>46223.81917953704</v>
+        <v>46223.652512870365</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>206</v>
@@ -4446,13 +4446,13 @@
         <v>209</v>
       </c>
       <c r="B53" s="8">
-        <v>46077.511973553235</v>
+        <v>46077.34530688658</v>
       </c>
       <c r="C53" s="8">
-        <v>46181.5844784838</v>
+        <v>46181.417811817126</v>
       </c>
       <c r="D53" s="8">
-        <v>46223.819175983794</v>
+        <v>46223.65250931713</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>210</v>
@@ -4509,13 +4509,13 @@
         <v>212</v>
       </c>
       <c r="B54" s="5">
-        <v>46077.51198193287</v>
+        <v>46077.345315266204</v>
       </c>
       <c r="C54" s="5">
-        <v>46181.5844847338</v>
+        <v>46181.41781806713</v>
       </c>
       <c r="D54" s="5">
-        <v>46223.81917170139</v>
+        <v>46223.652505034726</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>213</v>
@@ -4572,13 +4572,13 @@
         <v>215</v>
       </c>
       <c r="B55" s="8">
-        <v>46077.51201255787</v>
+        <v>46077.345345891204</v>
       </c>
       <c r="C55" s="8">
-        <v>46181.58491251158</v>
+        <v>46181.41824584491</v>
       </c>
       <c r="D55" s="8">
-        <v>46223.819168194445</v>
+        <v>46223.65250152777</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>157</v>
@@ -4635,13 +4635,13 @@
         <v>218</v>
       </c>
       <c r="B56" s="5">
-        <v>46077.512021215276</v>
+        <v>46077.34535454861</v>
       </c>
       <c r="C56" s="5">
-        <v>46181.58484026621</v>
+        <v>46181.41817359954</v>
       </c>
       <c r="D56" s="5">
-        <v>46223.81916162037</v>
+        <v>46223.652494953705</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>158</v>
@@ -4700,13 +4700,13 @@
         <v>220</v>
       </c>
       <c r="B57" s="8">
-        <v>46077.51202702546</v>
+        <v>46077.3453603588</v>
       </c>
       <c r="C57" s="8">
-        <v>46181.58575745371</v>
+        <v>46181.419090787036</v>
       </c>
       <c r="D57" s="8">
-        <v>46181.58575875</v>
+        <v>46181.419092083335</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>221</v>
@@ -4749,13 +4749,13 @@
         <v>223</v>
       </c>
       <c r="B58" s="5">
-        <v>46077.51207347222</v>
+        <v>46077.34540680556</v>
       </c>
       <c r="C58" s="5">
-        <v>46181.584975081016</v>
+        <v>46181.41830841435</v>
       </c>
       <c r="D58" s="5">
-        <v>46181.66365998842</v>
+        <v>46181.49699332176</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>224</v>
@@ -4814,13 +4814,13 @@
         <v>227</v>
       </c>
       <c r="B59" s="8">
-        <v>46077.51208324074</v>
+        <v>46077.34541657407</v>
       </c>
       <c r="C59" s="8">
-        <v>46181.585011284726</v>
+        <v>46181.418344618054</v>
       </c>
       <c r="D59" s="8">
-        <v>46223.81920950231</v>
+        <v>46223.65254283565</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>228</v>
@@ -4879,13 +4879,13 @@
         <v>230</v>
       </c>
       <c r="B60" s="5">
-        <v>46077.5120906713</v>
+        <v>46077.34542400463</v>
       </c>
       <c r="C60" s="5">
-        <v>46150.695240960646</v>
+        <v>46150.52857429398</v>
       </c>
       <c r="D60" s="5">
-        <v>46181.663659432874</v>
+        <v>46181.4969927662</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>231</v>
@@ -4944,13 +4944,13 @@
         <v>233</v>
       </c>
       <c r="B61" s="8">
-        <v>46077.512098148145</v>
+        <v>46077.34543148148</v>
       </c>
       <c r="C61" s="8">
-        <v>46181.58499498843</v>
+        <v>46181.41832832176</v>
       </c>
       <c r="D61" s="8">
-        <v>46181.663660543985</v>
+        <v>46181.496993877314</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>234</v>
@@ -5009,13 +5009,13 @@
         <v>236</v>
       </c>
       <c r="B62" s="5">
-        <v>46077.512106423615</v>
+        <v>46077.345439756944</v>
       </c>
       <c r="C62" s="5">
-        <v>46240.60840010417</v>
+        <v>46240.4417334375</v>
       </c>
       <c r="D62" s="5">
-        <v>46240.60840165509</v>
+        <v>46240.441734988424</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>237</v>
@@ -5058,13 +5058,13 @@
         <v>239</v>
       </c>
       <c r="B63" s="8">
-        <v>46077.512111296295</v>
+        <v>46077.34544462963</v>
       </c>
       <c r="C63" s="8">
-        <v>46240.607980057874</v>
+        <v>46240.4413133912</v>
       </c>
       <c r="D63" s="8">
-        <v>46240.60846284722</v>
+        <v>46240.44179618056</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>240</v>
@@ -5123,13 +5123,13 @@
         <v>243</v>
       </c>
       <c r="B64" s="5">
-        <v>46077.51211840278</v>
+        <v>46077.34545173611</v>
       </c>
       <c r="C64" s="5">
-        <v>46240.60799158565</v>
+        <v>46240.44132491898</v>
       </c>
       <c r="D64" s="5">
-        <v>46240.608487488425</v>
+        <v>46240.441820821754</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>244</v>

</xml_diff>